<commit_message>
touches on pivot chart
</commit_message>
<xml_diff>
--- a/Ocelotl4_territory_chart.xlsx
+++ b/Ocelotl4_territory_chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/locelotllopez_my_yearupunited_org/Documents/Documents/data_labs/Capstone_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{458B4B8A-A6F8-4DBB-AC8F-80550C9EADD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{458B4B8A-A6F8-4DBB-AC8F-80550C9EADD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DF6B064-8E72-49CD-812E-1B46D98632D2}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8B617B1-64C2-497B-84ED-0954870CB31D}"/>
+    <workbookView minimized="1" xWindow="1404" yWindow="1656" windowWidth="17280" windowHeight="8880" xr2:uid="{F8B617B1-64C2-497B-84ED-0954870CB31D}"/>
   </bookViews>
   <sheets>
     <sheet name="category_count_chart" sheetId="2" r:id="rId1"/>
@@ -1074,6 +1074,7 @@
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
+          <c:numFmt formatCode="#,##0.00" sourceLinked="0"/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -4535,6 +4536,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="#,##0.00" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>

</xml_diff>

<commit_message>
finished bonus questions and touched up my analysis
</commit_message>
<xml_diff>
--- a/Ocelotl4_territory_chart.xlsx
+++ b/Ocelotl4_territory_chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/locelotllopez_my_yearupunited_org/Documents/Documents/data_labs/Capstone_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{458B4B8A-A6F8-4DBB-AC8F-80550C9EADD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A49C4581-63A3-4C9A-B242-CC628664A9B7}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{458B4B8A-A6F8-4DBB-AC8F-80550C9EADD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6A6556B-91D8-459B-9531-F0DE89AA98DF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F8B617B1-64C2-497B-84ED-0954870CB31D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F8B617B1-64C2-497B-84ED-0954870CB31D}"/>
   </bookViews>
   <sheets>
     <sheet name="category_count_chart" sheetId="2" r:id="rId1"/>

</xml_diff>